<commit_message>
fix register, login, delete (user); hash code password; fix update_user otp, transfer otp
</commit_message>
<xml_diff>
--- a/data/logs.xlsx
+++ b/data/logs.xlsx
@@ -145,6 +145,93 @@
   </si>
   <si>
     <t>2025-03-25 21:46:01</t>
+  </si>
+  <si>
+    <t>Chuyển tiền thành công</t>
+  </si>
+  <si>
+    <t>2025-05-20 23:10:41</t>
+  </si>
+  <si>
+    <t>Nhận tiền</t>
+  </si>
+  <si>
+    <t>Chuyển điểm thành công</t>
+  </si>
+  <si>
+    <t>2025-05-21 09:27:13</t>
+  </si>
+  <si>
+    <t>Nhận điểm</t>
+  </si>
+  <si>
+    <t>2025-05-21 09:27:35</t>
+  </si>
+  <si>
+    <t>2025-05-21 09:31:27</t>
+  </si>
+  <si>
+    <t>2025-05-21 10:30:39</t>
+  </si>
+  <si>
+    <t>2025-05-21 11:07:10</t>
+  </si>
+  <si>
+    <t>2025-05-21 11:08:52</t>
+  </si>
+  <si>
+    <t>2025-05-21 11:22:26</t>
+  </si>
+  <si>
+    <t>2025-05-21 11:28:45</t>
+  </si>
+  <si>
+    <t>2025-05-21 11:30:45</t>
+  </si>
+  <si>
+    <t>2025-05-21 11:37:17</t>
+  </si>
+  <si>
+    <t>2025-05-21 11:41:39</t>
+  </si>
+  <si>
+    <t>Nạp điểm khi tạo tài khoản</t>
+  </si>
+  <si>
+    <t>2025-05-21 12:03:59</t>
+  </si>
+  <si>
+    <t>2025-05-21 12:07:23</t>
+  </si>
+  <si>
+    <t>2025-05-21 12:12:23</t>
+  </si>
+  <si>
+    <t>Trừ điểm để nạp tài khoản mới</t>
+  </si>
+  <si>
+    <t>2025-05-21 12:17:05</t>
+  </si>
+  <si>
+    <t>2025-05-21 12:19:55</t>
+  </si>
+  <si>
+    <t>2025-05-21 12:23:34</t>
+  </si>
+  <si>
+    <t>2025-05-21 12:24:51</t>
+  </si>
+  <si>
+    <t>2025-05-21 12:30:20</t>
+  </si>
+  <si>
+    <t>2025-05-21 12:34:16</t>
+  </si>
+  <si>
+    <t>2025-05-21 12:34:29</t>
+  </si>
+  <si>
+    <t>2025-05-21 13:37:15</t>
   </si>
 </sst>
 </file>
@@ -811,6 +898,1124 @@
         <v>39</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17">
+        <v>23394</v>
+      </c>
+      <c r="E17">
+        <v>22394</v>
+      </c>
+      <c r="F17">
+        <v>3</v>
+      </c>
+      <c r="G17">
+        <v>4</v>
+      </c>
+      <c r="H17" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>4</v>
+      </c>
+      <c r="C18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D18">
+        <v>2396</v>
+      </c>
+      <c r="E18">
+        <v>3396</v>
+      </c>
+      <c r="F18">
+        <v>3</v>
+      </c>
+      <c r="G18">
+        <v>4</v>
+      </c>
+      <c r="H18" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19">
+        <v>1000000</v>
+      </c>
+      <c r="E19">
+        <v>999000</v>
+      </c>
+      <c r="F19">
+        <v>2</v>
+      </c>
+      <c r="G19">
+        <v>10</v>
+      </c>
+      <c r="H19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>10</v>
+      </c>
+      <c r="C20" t="s">
+        <v>45</v>
+      </c>
+      <c r="D20">
+        <v>500</v>
+      </c>
+      <c r="E20">
+        <v>1500</v>
+      </c>
+      <c r="F20">
+        <v>2</v>
+      </c>
+      <c r="G20">
+        <v>10</v>
+      </c>
+      <c r="H20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>3</v>
+      </c>
+      <c r="C21" t="s">
+        <v>43</v>
+      </c>
+      <c r="D21">
+        <v>22394</v>
+      </c>
+      <c r="E21">
+        <v>22294</v>
+      </c>
+      <c r="F21">
+        <v>3</v>
+      </c>
+      <c r="G21">
+        <v>4</v>
+      </c>
+      <c r="H21" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>45</v>
+      </c>
+      <c r="D22">
+        <v>3396</v>
+      </c>
+      <c r="E22">
+        <v>3496</v>
+      </c>
+      <c r="F22">
+        <v>3</v>
+      </c>
+      <c r="G22">
+        <v>4</v>
+      </c>
+      <c r="H22" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>3</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>22294</v>
+      </c>
+      <c r="E23">
+        <v>21294</v>
+      </c>
+      <c r="F23">
+        <v>3</v>
+      </c>
+      <c r="G23">
+        <v>5</v>
+      </c>
+      <c r="H23" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>5</v>
+      </c>
+      <c r="C24" t="s">
+        <v>45</v>
+      </c>
+      <c r="D24">
+        <v>2395</v>
+      </c>
+      <c r="E24">
+        <v>3395</v>
+      </c>
+      <c r="F24">
+        <v>3</v>
+      </c>
+      <c r="G24">
+        <v>5</v>
+      </c>
+      <c r="H24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>3</v>
+      </c>
+      <c r="C25" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25">
+        <v>21294</v>
+      </c>
+      <c r="E25">
+        <v>20294</v>
+      </c>
+      <c r="F25">
+        <v>3</v>
+      </c>
+      <c r="G25">
+        <v>4</v>
+      </c>
+      <c r="H25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>45</v>
+      </c>
+      <c r="D26">
+        <v>3496</v>
+      </c>
+      <c r="E26">
+        <v>4496</v>
+      </c>
+      <c r="F26">
+        <v>3</v>
+      </c>
+      <c r="G26">
+        <v>4</v>
+      </c>
+      <c r="H26" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>2</v>
+      </c>
+      <c r="C27" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27">
+        <v>999000</v>
+      </c>
+      <c r="E27">
+        <v>998000</v>
+      </c>
+      <c r="F27">
+        <v>2</v>
+      </c>
+      <c r="G27">
+        <v>3</v>
+      </c>
+      <c r="H27" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>3</v>
+      </c>
+      <c r="C28" t="s">
+        <v>45</v>
+      </c>
+      <c r="D28">
+        <v>20294</v>
+      </c>
+      <c r="E28">
+        <v>21294</v>
+      </c>
+      <c r="F28">
+        <v>2</v>
+      </c>
+      <c r="G28">
+        <v>3</v>
+      </c>
+      <c r="H28" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29">
+        <v>998000</v>
+      </c>
+      <c r="E29">
+        <v>997000</v>
+      </c>
+      <c r="F29">
+        <v>2</v>
+      </c>
+      <c r="G29">
+        <v>3</v>
+      </c>
+      <c r="H29" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30" t="s">
+        <v>45</v>
+      </c>
+      <c r="D30">
+        <v>21294</v>
+      </c>
+      <c r="E30">
+        <v>22294</v>
+      </c>
+      <c r="F30">
+        <v>2</v>
+      </c>
+      <c r="G30">
+        <v>3</v>
+      </c>
+      <c r="H30" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>997000</v>
+      </c>
+      <c r="E31">
+        <v>996000</v>
+      </c>
+      <c r="F31">
+        <v>1</v>
+      </c>
+      <c r="G31">
+        <v>2</v>
+      </c>
+      <c r="H31" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>2</v>
+      </c>
+      <c r="C32" t="s">
+        <v>45</v>
+      </c>
+      <c r="D32">
+        <v>22294</v>
+      </c>
+      <c r="E32">
+        <v>23294</v>
+      </c>
+      <c r="F32">
+        <v>1</v>
+      </c>
+      <c r="G32">
+        <v>2</v>
+      </c>
+      <c r="H32" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>43</v>
+      </c>
+      <c r="D33">
+        <v>22294</v>
+      </c>
+      <c r="E33">
+        <v>22289</v>
+      </c>
+      <c r="F33">
+        <v>2</v>
+      </c>
+      <c r="G33">
+        <v>3</v>
+      </c>
+      <c r="H33" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>3</v>
+      </c>
+      <c r="C34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D34">
+        <v>4496</v>
+      </c>
+      <c r="E34">
+        <v>4501</v>
+      </c>
+      <c r="F34">
+        <v>2</v>
+      </c>
+      <c r="G34">
+        <v>3</v>
+      </c>
+      <c r="H34" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35" t="s">
+        <v>43</v>
+      </c>
+      <c r="D35">
+        <v>4501</v>
+      </c>
+      <c r="E35">
+        <v>4401</v>
+      </c>
+      <c r="F35">
+        <v>2</v>
+      </c>
+      <c r="G35">
+        <v>3</v>
+      </c>
+      <c r="H35" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>3</v>
+      </c>
+      <c r="C36" t="s">
+        <v>45</v>
+      </c>
+      <c r="D36">
+        <v>4496</v>
+      </c>
+      <c r="E36">
+        <v>4596</v>
+      </c>
+      <c r="F36">
+        <v>2</v>
+      </c>
+      <c r="G36">
+        <v>3</v>
+      </c>
+      <c r="H36" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>2</v>
+      </c>
+      <c r="C37" t="s">
+        <v>43</v>
+      </c>
+      <c r="D37">
+        <v>100000</v>
+      </c>
+      <c r="E37">
+        <v>99000</v>
+      </c>
+      <c r="F37">
+        <v>1</v>
+      </c>
+      <c r="G37">
+        <v>3</v>
+      </c>
+      <c r="H37" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>4</v>
+      </c>
+      <c r="C38" t="s">
+        <v>45</v>
+      </c>
+      <c r="D38">
+        <v>500</v>
+      </c>
+      <c r="E38">
+        <v>1500</v>
+      </c>
+      <c r="F38">
+        <v>1</v>
+      </c>
+      <c r="G38">
+        <v>3</v>
+      </c>
+      <c r="H38" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39" t="s">
+        <v>43</v>
+      </c>
+      <c r="D39">
+        <v>99000</v>
+      </c>
+      <c r="E39">
+        <v>98000</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="G39">
+        <v>1</v>
+      </c>
+      <c r="H39" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>45</v>
+      </c>
+      <c r="D40">
+        <v>99000</v>
+      </c>
+      <c r="E40">
+        <v>100000</v>
+      </c>
+      <c r="F40">
+        <v>1</v>
+      </c>
+      <c r="G40">
+        <v>1</v>
+      </c>
+      <c r="H40" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>13</v>
+      </c>
+      <c r="C41" t="s">
+        <v>56</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>500</v>
+      </c>
+      <c r="F41">
+        <v>1</v>
+      </c>
+      <c r="G41">
+        <v>12</v>
+      </c>
+      <c r="H41" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>14</v>
+      </c>
+      <c r="C42" t="s">
+        <v>56</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>500</v>
+      </c>
+      <c r="F42">
+        <v>1</v>
+      </c>
+      <c r="G42">
+        <v>13</v>
+      </c>
+      <c r="H42" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>15</v>
+      </c>
+      <c r="C43" t="s">
+        <v>56</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="E43">
+        <v>500</v>
+      </c>
+      <c r="F43">
+        <v>1</v>
+      </c>
+      <c r="G43">
+        <v>14</v>
+      </c>
+      <c r="H43" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>60</v>
+      </c>
+      <c r="D44">
+        <v>98500</v>
+      </c>
+      <c r="E44">
+        <v>98000</v>
+      </c>
+      <c r="F44">
+        <v>1</v>
+      </c>
+      <c r="G44">
+        <v>15</v>
+      </c>
+      <c r="H44" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>15</v>
+      </c>
+      <c r="C45" t="s">
+        <v>56</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45">
+        <v>500</v>
+      </c>
+      <c r="F45">
+        <v>1</v>
+      </c>
+      <c r="G45">
+        <v>15</v>
+      </c>
+      <c r="H45" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>2</v>
+      </c>
+      <c r="C46" t="s">
+        <v>43</v>
+      </c>
+      <c r="D46">
+        <v>98000</v>
+      </c>
+      <c r="E46">
+        <v>97000</v>
+      </c>
+      <c r="F46">
+        <v>1</v>
+      </c>
+      <c r="G46">
+        <v>2</v>
+      </c>
+      <c r="H46" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>3</v>
+      </c>
+      <c r="C47" t="s">
+        <v>45</v>
+      </c>
+      <c r="D47">
+        <v>500</v>
+      </c>
+      <c r="E47">
+        <v>1500</v>
+      </c>
+      <c r="F47">
+        <v>1</v>
+      </c>
+      <c r="G47">
+        <v>2</v>
+      </c>
+      <c r="H47" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>2</v>
+      </c>
+      <c r="C48" t="s">
+        <v>43</v>
+      </c>
+      <c r="D48">
+        <v>97000</v>
+      </c>
+      <c r="E48">
+        <v>96900</v>
+      </c>
+      <c r="F48">
+        <v>1</v>
+      </c>
+      <c r="G48">
+        <v>3</v>
+      </c>
+      <c r="H48" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49">
+        <v>4</v>
+      </c>
+      <c r="C49" t="s">
+        <v>45</v>
+      </c>
+      <c r="D49">
+        <v>1500</v>
+      </c>
+      <c r="E49">
+        <v>1600</v>
+      </c>
+      <c r="F49">
+        <v>1</v>
+      </c>
+      <c r="G49">
+        <v>3</v>
+      </c>
+      <c r="H49" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>43</v>
+      </c>
+      <c r="D50">
+        <v>1500</v>
+      </c>
+      <c r="E50">
+        <v>1499</v>
+      </c>
+      <c r="F50">
+        <v>2</v>
+      </c>
+      <c r="G50">
+        <v>3</v>
+      </c>
+      <c r="H50" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <v>4</v>
+      </c>
+      <c r="C51" t="s">
+        <v>45</v>
+      </c>
+      <c r="D51">
+        <v>1600</v>
+      </c>
+      <c r="E51">
+        <v>1601</v>
+      </c>
+      <c r="F51">
+        <v>2</v>
+      </c>
+      <c r="G51">
+        <v>3</v>
+      </c>
+      <c r="H51" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52">
+        <v>2</v>
+      </c>
+      <c r="C52" t="s">
+        <v>43</v>
+      </c>
+      <c r="D52">
+        <v>96900</v>
+      </c>
+      <c r="E52">
+        <v>96899</v>
+      </c>
+      <c r="F52">
+        <v>1</v>
+      </c>
+      <c r="G52">
+        <v>2</v>
+      </c>
+      <c r="H52" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53">
+        <v>3</v>
+      </c>
+      <c r="C53" t="s">
+        <v>45</v>
+      </c>
+      <c r="D53">
+        <v>1499</v>
+      </c>
+      <c r="E53">
+        <v>1500</v>
+      </c>
+      <c r="F53">
+        <v>1</v>
+      </c>
+      <c r="G53">
+        <v>2</v>
+      </c>
+      <c r="H53" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>60</v>
+      </c>
+      <c r="D54">
+        <v>96899</v>
+      </c>
+      <c r="E54">
+        <v>96399</v>
+      </c>
+      <c r="F54">
+        <v>1</v>
+      </c>
+      <c r="G54">
+        <v>16</v>
+      </c>
+      <c r="H54" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55">
+        <v>16</v>
+      </c>
+      <c r="C55" t="s">
+        <v>56</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55">
+        <v>500</v>
+      </c>
+      <c r="F55">
+        <v>1</v>
+      </c>
+      <c r="G55">
+        <v>16</v>
+      </c>
+      <c r="H55" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56">
+        <v>2</v>
+      </c>
+      <c r="C56" t="s">
+        <v>43</v>
+      </c>
+      <c r="D56">
+        <v>96399</v>
+      </c>
+      <c r="E56">
+        <v>96398</v>
+      </c>
+      <c r="F56">
+        <v>1</v>
+      </c>
+      <c r="G56">
+        <v>3</v>
+      </c>
+      <c r="H56" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57">
+        <v>4</v>
+      </c>
+      <c r="C57" t="s">
+        <v>45</v>
+      </c>
+      <c r="D57">
+        <v>1601</v>
+      </c>
+      <c r="E57">
+        <v>1602</v>
+      </c>
+      <c r="F57">
+        <v>1</v>
+      </c>
+      <c r="G57">
+        <v>3</v>
+      </c>
+      <c r="H57" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
+      </c>
+      <c r="C58" t="s">
+        <v>60</v>
+      </c>
+      <c r="D58">
+        <v>96398</v>
+      </c>
+      <c r="E58">
+        <v>95898</v>
+      </c>
+      <c r="F58">
+        <v>1</v>
+      </c>
+      <c r="G58">
+        <v>17</v>
+      </c>
+      <c r="H58" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59">
+        <v>17</v>
+      </c>
+      <c r="C59" t="s">
+        <v>56</v>
+      </c>
+      <c r="D59">
+        <v>0</v>
+      </c>
+      <c r="E59">
+        <v>500</v>
+      </c>
+      <c r="F59">
+        <v>1</v>
+      </c>
+      <c r="G59">
+        <v>17</v>
+      </c>
+      <c r="H59" t="s">
+        <v>68</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>